<commit_message>
chore: versiona a planilha de custos de LLM e adiciona .gitattributes
Acrescenta docs/mcp-redmine-costs.xlsx ao controle de versao, com uma
excecao ao padrao *.xlsx do .gitignore, e registra a sessao do Cowork
que implementou o suporte a .env: claude-opus-5, US$ 18,94 pelos precos
oficiais da Claude Platform.

O .gitattributes trata os formatos Office como binarios e fixa LF como
quebra de linha no repositorio.
</commit_message>
<xml_diff>
--- a/docs/mcp-redmine-costs.xlsx
+++ b/docs/mcp-redmine-costs.xlsx
@@ -975,19 +975,19 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>247</v>
+        <v>329</v>
       </c>
       <c r="H7" t="n">
-        <v>87839</v>
+        <v>119254</v>
       </c>
       <c r="I7" t="n">
-        <v>10998938</v>
+        <v>17460397</v>
       </c>
       <c r="J7" t="n">
-        <v>609279</v>
+        <v>722754</v>
       </c>
       <c r="K7" t="n">
-        <v>13.7895</v>
+        <v>18.9407</v>
       </c>
       <c r="L7">
         <f>ROUNDUP($K7*Config!$B$1,2)</f>
@@ -995,7 +995,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Suporte a .env no mcp-redmine (config.py, testes, docs) + commit</t>
+          <t>Suporte a .env no mcp-redmine (config.py, testes, docs), .gitattributes e planilha de custos</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">

</xml_diff>